<commit_message>
fix: firmware/alias names: nullptr, if IOs are reconfgured
</commit_message>
<xml_diff>
--- a/docs_raw/spannungsberechnung rc.xlsx
+++ b/docs_raw/spannungsberechnung rc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stefan\Documents\ft\ftSwarm3\ftSwarm\docs_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B21786A-1D79-454D-8B87-086EDEE58AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06ED3E11-4D7D-48BF-A857-AD61F0A3817B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F51EC718-0BE4-43DA-97F7-C878CB2657B1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F51EC718-0BE4-43DA-97F7-C878CB2657B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>

</xml_diff>